<commit_message>
se actualizo el pdf
</commit_message>
<xml_diff>
--- a/spreadsheet/Clara_AWS_Cost_Optimization_Model.xlsx
+++ b/spreadsheet/Clara_AWS_Cost_Optimization_Model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\AWS Cost Optimization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\AWS Cost Optimization\spreadsheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A6E0403-4EDB-4873-BC47-DB819825B139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C109CBF8-303B-4798-9829-A23BB521B1C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14070" yWindow="375" windowWidth="17655" windowHeight="15750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14070" yWindow="375" windowWidth="17655" windowHeight="15750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Current_Costs" sheetId="1" r:id="rId1"/>
@@ -1133,26 +1133,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1296,6 +1276,19 @@
             </c:numRef>
           </c:val>
           <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-8331-4236-98CB-D8A54B1134F7}"/>
             </c:ext>
@@ -1436,6 +1429,19 @@
             </c:numRef>
           </c:val>
           <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-8331-4236-98CB-D8A54B1134F7}"/>
             </c:ext>
@@ -1576,6 +1582,19 @@
             </c:numRef>
           </c:val>
           <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-8331-4236-98CB-D8A54B1134F7}"/>
             </c:ext>
@@ -1650,26 +1669,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1756,26 +1755,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1871,570 +1850,6 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="202">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="800" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
-    <cs:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="22225" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1600" b="1" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="800" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
@@ -2444,7 +1859,7 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>133349</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5572125" cy="4800601"/>
+    <xdr:ext cx="7620000" cy="4800601"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -2469,10 +1884,6 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3110,6 +2521,24 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C7">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E2:E7">
     <cfRule type="dataBar" priority="1">
       <dataBar>
@@ -3122,26 +2551,6 @@
           <x14:id>{4B81207E-6D84-4620-8A91-A74E08B3D4E1}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C7">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFF7128"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C7">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFF7128"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
se ajusto el excel
</commit_message>
<xml_diff>
--- a/spreadsheet/Clara_AWS_Cost_Optimization_Model.xlsx
+++ b/spreadsheet/Clara_AWS_Cost_Optimization_Model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\AWS Cost Optimization\spreadsheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C109CBF8-303B-4798-9829-A23BB521B1C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EAB01DA-FD4E-4837-B49C-924977EA3001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14070" yWindow="375" windowWidth="17655" windowHeight="15750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11385" yWindow="375" windowWidth="20340" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Current_Costs" sheetId="1" r:id="rId1"/>
     <sheet name="02_Optimization_Model" sheetId="2" r:id="rId2"/>
     <sheet name="03_Assumptions" sheetId="3" r:id="rId3"/>
+    <sheet name="04_Formula_Logic" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="90">
   <si>
     <t>Service</t>
   </si>
@@ -118,92 +119,208 @@
     <t>Monthly Savings</t>
   </si>
   <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>Assumption</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>35% reduction</t>
+  </si>
+  <si>
+    <t>CPU at 30% indicates overprovisioning</t>
+  </si>
+  <si>
+    <t>30% reduction</t>
+  </si>
+  <si>
+    <t>No autoscaling</t>
+  </si>
+  <si>
+    <t>Unattached volumes + snapshots</t>
+  </si>
+  <si>
+    <t>40% reduction</t>
+  </si>
+  <si>
+    <t>80% in Standard storage</t>
+  </si>
+  <si>
+    <t>Optimization Levers</t>
+  </si>
+  <si>
+    <t>Lever</t>
+  </si>
+  <si>
+    <t>Applies To</t>
+  </si>
+  <si>
+    <t>Rightsizing</t>
+  </si>
+  <si>
+    <t>EC2, EKS</t>
+  </si>
+  <si>
+    <t>Autoscaling</t>
+  </si>
+  <si>
+    <t>Storage Tiering</t>
+  </si>
+  <si>
+    <t>Cleanup</t>
+  </si>
+  <si>
+    <t>Savings Plans</t>
+  </si>
+  <si>
     <t>Total Savings %</t>
   </si>
   <si>
-    <t>Area</t>
-  </si>
-  <si>
-    <t>Assumption</t>
-  </si>
-  <si>
-    <t>Reason</t>
-  </si>
-  <si>
-    <t>35% reduction</t>
-  </si>
-  <si>
-    <t>CPU at 30% indicates overprovisioning</t>
-  </si>
-  <si>
-    <t>30% reduction</t>
-  </si>
-  <si>
-    <t>No autoscaling</t>
-  </si>
-  <si>
-    <t>Unattached volumes + snapshots</t>
-  </si>
-  <si>
-    <t>40% reduction</t>
-  </si>
-  <si>
-    <t>80% in Standard storage</t>
-  </si>
-  <si>
-    <t>10% reduction</t>
-  </si>
-  <si>
-    <t>Conservative estimate</t>
-  </si>
-  <si>
-    <t>5% reduction</t>
-  </si>
-  <si>
-    <t>Already efficient</t>
-  </si>
-  <si>
-    <t>Optimization Levers</t>
-  </si>
-  <si>
-    <t>Lever</t>
-  </si>
-  <si>
-    <t>Applies To</t>
-  </si>
-  <si>
-    <t>Rightsizing</t>
-  </si>
-  <si>
-    <t>EC2, EKS</t>
-  </si>
-  <si>
-    <t>Autoscaling</t>
-  </si>
-  <si>
-    <t>Storage Tiering</t>
-  </si>
-  <si>
-    <t>Cleanup</t>
-  </si>
-  <si>
-    <t>Savings Plans</t>
+    <t>Executive Model Note:</t>
+  </si>
+  <si>
+    <t>This model presents the primary validated savings estimate used in the executive report. RDS and Lambda are treated as future optimization opportunities and are not included in the $70,000 monthly savings estimate. This keeps the recommendation conservative and aligned with the technical assessment deliverables.</t>
+  </si>
+  <si>
+    <t>0% reduction</t>
+  </si>
+  <si>
+    <t>Future opportunity; reserved capacity and storage optimization require workload validation</t>
+  </si>
+  <si>
+    <t>Future opportunity; memory and duration tuning after observability review</t>
+  </si>
+  <si>
+    <t>Formula / Assumption</t>
+  </si>
+  <si>
+    <t>Result / Explanation</t>
+  </si>
+  <si>
+    <t>Total AWS Monthly Spend</t>
+  </si>
+  <si>
+    <t>User-provided baseline</t>
+  </si>
+  <si>
+    <t>EC2 Current Cost</t>
+  </si>
+  <si>
+    <t>$250,000 × 40%</t>
+  </si>
+  <si>
+    <t>EBS Current Cost</t>
+  </si>
+  <si>
+    <t>$250,000 × 20%</t>
+  </si>
+  <si>
+    <t>RDS Current Cost</t>
+  </si>
+  <si>
+    <t>$250,000 × 15%</t>
+  </si>
+  <si>
+    <t>S3 Current Cost</t>
+  </si>
+  <si>
+    <t>$250,000 × 10%</t>
+  </si>
+  <si>
+    <t>EKS Current Cost</t>
+  </si>
+  <si>
+    <t>Lambda Current Cost</t>
+  </si>
+  <si>
+    <t>$250,000 × 5%</t>
+  </si>
+  <si>
+    <t>EC2 Optimization</t>
+  </si>
+  <si>
+    <t>$100,000 × 35%</t>
+  </si>
+  <si>
+    <t>$35,000 savings</t>
+  </si>
+  <si>
+    <t>EBS Optimization</t>
+  </si>
+  <si>
+    <t>$50,000 × 35%</t>
+  </si>
+  <si>
+    <t>$17,500 savings</t>
+  </si>
+  <si>
+    <t>RDS Optimization</t>
+  </si>
+  <si>
+    <t>$37,500 × 0%</t>
+  </si>
+  <si>
+    <t>No savings applied in executive model; future opportunity</t>
+  </si>
+  <si>
+    <t>S3 Optimization</t>
+  </si>
+  <si>
+    <t>$25,000 × 40%</t>
+  </si>
+  <si>
+    <t>$10,000 savings</t>
+  </si>
+  <si>
+    <t>EKS Optimization</t>
+  </si>
+  <si>
+    <t>$25,000 × 30%</t>
+  </si>
+  <si>
+    <t>$7,500 savings</t>
+  </si>
+  <si>
+    <t>Lambda Optimization</t>
+  </si>
+  <si>
+    <t>$12,500 × 0%</t>
+  </si>
+  <si>
+    <t>Total Estimated Savings</t>
+  </si>
+  <si>
+    <t>SUM(EC2, EBS, S3, EKS savings)</t>
+  </si>
+  <si>
+    <t>Optimized Monthly Spend</t>
+  </si>
+  <si>
+    <t>$250,000 - $70,000</t>
+  </si>
+  <si>
+    <t>Savings Percentage</t>
+  </si>
+  <si>
+    <t>$70,000 / $250,000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -215,8 +332,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -241,19 +356,21 @@
       <sz val="11"/>
       <color rgb="FF548235"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF548235"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F2937"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,58 +380,59 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD6DCE4"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2E75B6"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF548235"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFD6E3F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7ED"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="25">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -359,21 +477,6 @@
         <color rgb="FFD9D9D9"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="double">
-        <color rgb="FF1F4E79"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -548,66 +651,6 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FF2E75B6"/>
       </left>
       <right style="thin">
@@ -724,175 +767,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFD9E2EC"/>
       </left>
       <right style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFD9E2EC"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FFD9E2EC"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1F4E79"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1F4E79"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF1F4E79"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF1F4E79"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1F4E79"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF1F4E79"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF1F4E79"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF1F4E79"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF1F4E79"/>
+        <color rgb="FFD9E2EC"/>
       </bottom>
       <diagonal/>
     </border>
@@ -900,56 +784,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -957,104 +842,121 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="38" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="4" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1066,14 +968,13 @@
         <color rgb="FFC65911"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFCE4D6"/>
+        <patternFill>
+          <bgColor indexed="64"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1105,19 +1006,6 @@
           <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
               <a:t>Current vs Optimized Cost</a:t>
@@ -1125,7 +1013,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="1"/>
+      <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -1133,6 +1021,14 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1205,20 +1101,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1276,21 +1159,8 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
-              <c14:invertSolidFillFmt>
-                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c14:spPr>
-              </c14:invertSolidFillFmt>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8331-4236-98CB-D8A54B1134F7}"/>
+              <c16:uniqueId val="{00000000-28F3-4673-83AF-A03191A758F9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1358,20 +1228,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1420,30 +1277,17 @@
                   <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.05</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
-              <c14:invertSolidFillFmt>
-                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c14:spPr>
-              </c14:invertSolidFillFmt>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8331-4236-98CB-D8A54B1134F7}"/>
+              <c16:uniqueId val="{00000001-28F3-4673-83AF-A03191A758F9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1511,20 +1355,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1573,30 +1404,17 @@
                   <c:v>15000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>33750</c:v>
+                  <c:v>37500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11875</c:v>
+                  <c:v>12500</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
-              <c14:invertSolidFillFmt>
-                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c14:spPr>
-              </c14:invertSolidFillFmt>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-8331-4236-98CB-D8A54B1134F7}"/>
+              <c16:uniqueId val="{00000002-28F3-4673-83AF-A03191A758F9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1611,11 +1429,11 @@
         </c:dLbls>
         <c:gapWidth val="444"/>
         <c:overlap val="-90"/>
-        <c:axId val="10"/>
-        <c:axId val="100"/>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10"/>
+        <c:axId val="48650112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1641,19 +1459,6 @@
               <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
                   <a:t>Service</a:t>
@@ -1661,7 +1466,7 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="1"/>
+          <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -1669,6 +1474,14 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1707,15 +1520,15 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="100"/>
+        <c:crossAx val="48672768"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="1"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="100"/>
+        <c:axId val="48672768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1727,19 +1540,6 @@
               <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
                   <a:t>USD</a:t>
@@ -1747,7 +1547,7 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="1"/>
+          <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -1755,12 +1555,20 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
         </c:title>
         <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="10"/>
+        <c:crossAx val="48650112"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1774,16 +1582,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.25206259259259262"/>
-          <c:y val="6.1148148148148146E-2"/>
-          <c:w val="0.48511528366646478"/>
-          <c:h val="4.464316030430357E-2"/>
-        </c:manualLayout>
-      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1814,7 +1612,7 @@
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
+    <c:dispBlanksAs val="zero"/>
     <c:showDLblsOverMax val="1"/>
   </c:chart>
   <c:spPr>
@@ -1850,19 +1648,583 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="202">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="800" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+    <cs:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="22225" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="800" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>133349</xdr:rowOff>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>104774</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7620000" cy="4800601"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="2" name="Chart">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
@@ -1887,7 +2249,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1929,72 +2291,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2002,55 +2306,15 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="dk1"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="accent1"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -2059,13 +2323,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2099,24 +2363,13 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2142,7 +2395,7 @@
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2184,157 +2437,157 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="23">
+      <c r="B2" s="20">
         <v>100000</v>
       </c>
-      <c r="C2" s="28">
+      <c r="C2" s="25">
         <f t="shared" ref="C2:C7" si="0">B2/$B$8</f>
         <v>0.4</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="24">
+      <c r="B3" s="21">
         <v>50000</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="26">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="25">
+      <c r="B4" s="22">
         <v>37500</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="27">
         <f t="shared" si="0"/>
         <v>0.15</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="21">
         <v>25000</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="26">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="22">
         <v>25000</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="27">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="23">
         <v>12500</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="28">
         <f t="shared" si="0"/>
         <v>0.05</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="24">
         <f>SUM(B2:B7)</f>
         <v>250000</v>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="29">
         <f>1</f>
         <v>1</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="10"/>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="33">
+      <c r="B12" s="30">
         <v>500</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="31">
         <v>0.6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="35">
+      <c r="B14" s="32">
         <v>0.3</v>
       </c>
     </row>
@@ -2344,7 +2597,7 @@
       <formula>NOT(ISERROR(SEARCH("Overprovisioned",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2353,174 +2606,186 @@
   <sheetPr>
     <tabColor rgb="FF548235"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="40.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="5" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="33" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="43">
+      <c r="B2" s="35">
         <v>100000</v>
       </c>
-      <c r="C2" s="47">
+      <c r="C2" s="36">
         <v>0.35</v>
       </c>
-      <c r="D2" s="43">
-        <f t="shared" ref="D2:D7" si="0">B2*(1-C2)</f>
+      <c r="D2" s="35">
+        <f t="shared" ref="D2:D7" si="0">B2-E2</f>
         <v>65000</v>
       </c>
-      <c r="E2" s="67">
-        <f t="shared" ref="E2:E7" si="1">B2-D2</f>
+      <c r="E2" s="37">
+        <f t="shared" ref="E2:E7" si="1">B2*C2</f>
         <v>35000</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="44">
+      <c r="B3" s="39">
         <v>25000</v>
       </c>
-      <c r="C3" s="48">
+      <c r="C3" s="40">
         <v>0.3</v>
       </c>
-      <c r="D3" s="44">
+      <c r="D3" s="39">
         <f t="shared" si="0"/>
         <v>17500</v>
       </c>
-      <c r="E3" s="68">
+      <c r="E3" s="37">
         <f t="shared" si="1"/>
         <v>7500</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="45">
+      <c r="B4" s="35">
         <v>50000</v>
       </c>
-      <c r="C4" s="49">
+      <c r="C4" s="36">
         <v>0.35</v>
       </c>
-      <c r="D4" s="45">
+      <c r="D4" s="35">
         <f t="shared" si="0"/>
         <v>32500</v>
       </c>
-      <c r="E4" s="68">
+      <c r="E4" s="37">
         <f t="shared" si="1"/>
         <v>17500</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="39">
         <v>25000</v>
       </c>
-      <c r="C5" s="48">
+      <c r="C5" s="40">
         <v>0.4</v>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="39">
         <f t="shared" si="0"/>
         <v>15000</v>
       </c>
-      <c r="E5" s="68">
+      <c r="E5" s="37">
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="45">
+      <c r="B6" s="35">
         <v>37500</v>
       </c>
-      <c r="C6" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="D6" s="45">
+      <c r="C6" s="36">
+        <v>0</v>
+      </c>
+      <c r="D6" s="35">
         <f t="shared" si="0"/>
-        <v>33750</v>
-      </c>
-      <c r="E6" s="68">
+        <v>37500</v>
+      </c>
+      <c r="E6" s="37">
         <f t="shared" si="1"/>
-        <v>3750</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="46">
+      <c r="B7" s="39">
         <v>12500</v>
       </c>
-      <c r="C7" s="50">
-        <v>0.05</v>
-      </c>
-      <c r="D7" s="46">
+      <c r="C7" s="40">
+        <v>0</v>
+      </c>
+      <c r="D7" s="39">
         <f t="shared" si="0"/>
-        <v>11875</v>
-      </c>
-      <c r="E7" s="69">
+        <v>12500</v>
+      </c>
+      <c r="E7" s="37">
         <f t="shared" si="1"/>
-        <v>625</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="70">
+      <c r="B8" s="42">
         <f>SUM(B2:B7)</f>
         <v>250000</v>
       </c>
-      <c r="C8" s="71"/>
-      <c r="D8" s="70">
+      <c r="C8" s="44"/>
+      <c r="D8" s="42">
         <f>SUM(D2:D7)</f>
-        <v>175625</v>
-      </c>
-      <c r="E8" s="72">
+        <v>180000</v>
+      </c>
+      <c r="E8" s="43">
         <f>SUM(E2:E7)</f>
-        <v>74375</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="42">
+      <c r="A10" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="46">
         <f>E8/B8</f>
-        <v>0.29749999999999999</v>
-      </c>
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="68" customFormat="1" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="69" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="70" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B12:E12"/>
+  </mergeCells>
   <conditionalFormatting sqref="C2:C7">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -2552,18 +2817,37 @@
         </ext>
       </extLst>
     </cfRule>
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{4B81207E-6D84-4620-8A91-A74E08B3D4E1}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{4B81207E-6D84-4620-8A91-A74E08B3D4E1}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" direction="leftToRight" negativeBarColorSameAsPositive="1" axisPosition="none">
+            <x14:dataBar minLength="0" maxLength="100" negativeBarColorSameAsPositive="1" axisPosition="none">
+              <x14:cfvo type="min"/>
+              <x14:cfvo type="max"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <x14:cfRule type="dataBar" id="{4B81207E-6D84-4620-8A91-A74E08B3D4E1}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarColorSameAsPositive="1">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
               <x14:borderColor rgb="FF548235"/>
+              <x14:axisColor auto="1"/>
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>E2:E7</xm:sqref>
@@ -2582,142 +2866,360 @@
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
-    <col min="3" max="3" width="47.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="3" max="3" width="59.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:3" s="68" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="55" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="15" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="47" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="48" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="C2" s="47" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="49" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="49" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="47" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="49"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+    </row>
+    <row r="9" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="49"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="53" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="49"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="54" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="49"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="49"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="49"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="47" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="59" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="51" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
-        <v>12</v>
+      <c r="C15" s="49"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="55" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="55" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="58">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="59" t="s">
+        <v>56</v>
       </c>
       <c r="B3" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="52" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="61" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="53" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="40" t="s">
-        <v>10</v>
+        <v>57</v>
+      </c>
+      <c r="C3" s="61">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="57" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="58">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="59" t="s">
+        <v>60</v>
       </c>
       <c r="B5" s="60" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="52" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="61" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="54" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="62" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="55" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="56" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="63" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="64" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="57" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="65" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="64" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="58" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" s="66" t="s">
-        <v>4</v>
+        <v>61</v>
+      </c>
+      <c r="C5" s="61">
+        <v>37500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="56" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="58">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="59" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="60" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="61">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="57" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="58">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="59" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="62" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="56" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="57" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="60" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="62" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="56" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="57" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="60" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="62" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="57" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="63" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="65" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" s="66">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="64" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="65" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="66">
+        <v>180000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="64" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="67">
+        <v>0.28000000000000003</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>